<commit_message>
Clarify matching output change
</commit_message>
<xml_diff>
--- a/outputs/安排结果_第一轮.xlsx
+++ b/outputs/安排结果_第一轮.xlsx
@@ -468,12 +468,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>F3, F4, M1, M2</t>
+          <t>F2, F5, M5, M7</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>F3(高若曦), F4(梁欣怡), M1(赵浩然), M2(钱宇轩)</t>
+          <t>F2(何诗涵), F5(谢梦瑶), M5(周嘉铭), M7(郑明轩)</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -492,22 +492,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>F2, F6, M3, M7</t>
+          <t>F4, F6, M1, M2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>F2(何诗涵), F6(宋可欣), M3(孙子涵), M7(郑明轩)</t>
+          <t>F4(梁欣怡), F6(宋可欣), M1(赵浩然), M2(钱宇轩)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -516,22 +516,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>F7, F8, M4, M9</t>
+          <t>F1, F8, M6, M8</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>F7(唐婉清), F8(曹雅楠/原F9), M4(李俊熙), M9(冯博文)</t>
+          <t>F1(林雨桐), F8(曹雅楠/原F9), M6(吴泽宇), M8(王景辰)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -540,22 +540,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>F1, F9, M10, M6</t>
+          <t>F3, F7, M4, M9</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F1(林雨桐), F9(彭思妍/原F10), M10(陈奕辰), M6(吴泽宇)</t>
+          <t>F3(高若曦), F7(唐婉清), M4(李俊熙), M9(冯博文)</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>7</v>
       </c>
       <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
         <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -564,16 +564,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>F5, M5, M8</t>
+          <t>F9, M10, M3</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>F5(谢梦瑶), M5(周嘉铭), M8(王景辰)</t>
+          <t>F9(彭思妍/原F10), M10(陈奕辰), M3(孙子涵)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -644,22 +644,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>F3(高若曦)</t>
+          <t>M5(周嘉铭)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>M2(钱宇轩)</t>
+          <t>F2(何诗涵)</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -677,22 +677,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M1(赵浩然)</t>
+          <t>M7(郑明轩)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>F4(梁欣怡)</t>
+          <t>F2(何诗涵)</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -710,22 +710,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>F4(梁欣怡)</t>
+          <t>F5(谢梦瑶)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>M2(钱宇轩)</t>
+          <t>M5(周嘉铭)</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -753,12 +753,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>M3(孙子涵)</t>
+          <t>M1(赵浩然)</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -776,22 +776,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>M7(郑明轩)</t>
+          <t>M1(赵浩然)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>F2(何诗涵)</t>
+          <t>F4(梁欣怡)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -804,36 +804,36 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>单向喜欢</t>
+          <t>互相喜欢</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>M7(郑明轩)</t>
+          <t>F4(梁欣怡)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>F6</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>F6(宋可欣)</t>
+          <t>M2(钱宇轩)</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -842,22 +842,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>M3(孙子涵)</t>
+          <t>M6(吴泽宇)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F8</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>F2(何诗涵)</t>
+          <t>F8(曹雅楠/原F9)</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>F8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>M4(李俊熙)</t>
+          <t>F8(曹雅楠/原F9)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>F8(曹雅楠/原F9)</t>
+          <t>M8(王景辰)</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -903,36 +903,36 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>单向喜欢</t>
+          <t>互相喜欢</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>F7(唐婉清)</t>
+          <t>F1(林雨桐)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>M4(李俊熙)</t>
+          <t>M6(吴泽宇)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -941,22 +941,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>M9(冯博文)</t>
+          <t>M4(李俊熙)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>F7(唐婉清)</t>
+          <t>F3(高若曦)</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -965,7 +965,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -974,22 +974,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>F8(曹雅楠/原F9)</t>
+          <t>F7(唐婉清)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>M9(冯博文)</t>
+          <t>M4(李俊熙)</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -1002,31 +1002,31 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>互相喜欢</t>
+          <t>单向喜欢</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>F1(林雨桐)</t>
+          <t>M9(冯博文)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>M6(吴泽宇)</t>
+          <t>F7(唐婉清)</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1035,31 +1035,31 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>互相喜欢</t>
+          <t>单向喜欢</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>F9</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>F9(彭思妍/原F10)</t>
+          <t>M9(冯博文)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>M10(陈奕辰)</t>
+          <t>F3(高若曦)</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1073,22 +1073,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>F9</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>F5(谢梦瑶)</t>
+          <t>F9(彭思妍/原F10)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>M8(王景辰)</t>
+          <t>M3(孙子涵)</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -1106,22 +1106,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>F9</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>F5(谢梦瑶)</t>
+          <t>F9(彭思妍/原F10)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>M5(周嘉铭)</t>
+          <t>M10(陈奕辰)</t>
         </is>
       </c>
       <c r="G16" t="n">

</xml_diff>